<commit_message>
zhao tool not found
</commit_message>
<xml_diff>
--- a/assignment3/Results.xlsx
+++ b/assignment3/Results.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gostg\Documents\vscode\470\CMPT470-Future-Buisness-Majors\assignment3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kylen\gth842\cmpt470-a2\repo\assignment3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1ABB98B-E3F2-4280-831B-FB1E02FC4937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F24208E9-3FFD-48F9-B3C2-E71ED8D6E660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="51">
   <si>
     <t>Tool ID</t>
   </si>
@@ -172,6 +172,12 @@
   </si>
   <si>
     <t>Could not get the tool to work due to incorrect parsing logic</t>
+  </si>
+  <si>
+    <t>https://anonymous.4open.science/r/ECScan</t>
+  </si>
+  <si>
+    <t>Dead Artifact</t>
   </si>
 </sst>
 </file>
@@ -237,7 +243,7 @@
       <family val="3"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -253,6 +259,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -331,7 +343,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -356,7 +368,11 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -644,24 +660,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="46.85546875" customWidth="1"/>
-    <col min="2" max="2" width="15.85546875" customWidth="1"/>
+    <col min="1" max="1" width="46.88671875" customWidth="1"/>
+    <col min="2" max="2" width="15.88671875" customWidth="1"/>
     <col min="3" max="3" width="44" customWidth="1"/>
-    <col min="4" max="4" width="19.5703125" customWidth="1"/>
-    <col min="5" max="5" width="17.28515625" customWidth="1"/>
-    <col min="6" max="6" width="10.28515625" customWidth="1"/>
-    <col min="8" max="8" width="15.42578125" customWidth="1"/>
+    <col min="4" max="4" width="19.5546875" customWidth="1"/>
+    <col min="5" max="5" width="17.33203125" customWidth="1"/>
+    <col min="6" max="6" width="10.33203125" customWidth="1"/>
+    <col min="8" max="8" width="15.44140625" customWidth="1"/>
     <col min="9" max="9" width="16" customWidth="1"/>
-    <col min="10" max="10" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="24.7109375" customWidth="1"/>
-    <col min="13" max="13" width="15.140625" customWidth="1"/>
-    <col min="14" max="14" width="52.140625" customWidth="1"/>
+    <col min="12" max="12" width="24.6640625" customWidth="1"/>
+    <col min="13" max="13" width="15.109375" customWidth="1"/>
+    <col min="14" max="14" width="52.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -705,7 +721,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>27</v>
       </c>
@@ -747,7 +763,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>29</v>
       </c>
@@ -791,45 +807,47 @@
         <v>48</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
+    <row r="4" spans="1:14" s="26" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="3" t="s">
+      <c r="D4" s="24"/>
+      <c r="E4" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1" t="s">
+      <c r="F4" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I4" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="J4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N4" s="10" t="s">
+      <c r="J4" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="M4" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="N4" s="22" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>33</v>
       </c>
@@ -867,7 +885,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
         <v>35</v>
       </c>
@@ -905,34 +923,25 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C7" s="22"/>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="22"/>
-      <c r="I7" s="22"/>
-      <c r="J7" s="22"/>
-      <c r="K7" s="22"/>
-      <c r="L7" s="22"/>
-      <c r="M7" s="22"/>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C9" s="19" t="s">
         <v>40</v>
       </c>
       <c r="D9" s="20" t="s">
         <v>41</v>
       </c>
+      <c r="E9" s="26" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C10" s="17" t="s">
         <v>43</v>
       </c>
       <c r="D10" s="18" t="s">
         <v>42</v>
       </c>
+      <c r="E10" s="26"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updates to zhao and xcode
</commit_message>
<xml_diff>
--- a/assignment3/Results.xlsx
+++ b/assignment3/Results.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kylen\gth842\cmpt470-a2\repo\assignment3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F24208E9-3FFD-48F9-B3C2-E71ED8D6E660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0967497-04BF-4D5D-BB66-ED55BCBD76E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="58">
   <si>
     <t>Tool ID</t>
   </si>
@@ -96,9 +96,6 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>What is the problem/ why it didnt run,, what is tried</t>
-  </si>
-  <si>
     <t>Semantic Clones</t>
   </si>
   <si>
@@ -178,13 +175,37 @@
   </si>
   <si>
     <t>Dead Artifact</t>
+  </si>
+  <si>
+    <t>Windows 11 (N/A)</t>
+  </si>
+  <si>
+    <t>TES D</t>
+  </si>
+  <si>
+    <t>Future_Buisness_Majors_Xcode</t>
+  </si>
+  <si>
+    <t>Xcode</t>
+  </si>
+  <si>
+    <t>No working link exists</t>
+  </si>
+  <si>
+    <t>Github repo is expired, wayback did not crawl in time</t>
+  </si>
+  <si>
+    <t>93.7 (varies)</t>
+  </si>
+  <si>
+    <t>89.1 (varies)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -235,12 +256,6 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Consolas"/>
-      <family val="3"/>
     </font>
   </fonts>
   <fills count="5">
@@ -343,17 +358,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -365,14 +377,21 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -659,74 +678,75 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="46.88671875" customWidth="1"/>
     <col min="2" max="2" width="15.88671875" customWidth="1"/>
     <col min="3" max="3" width="44" customWidth="1"/>
-    <col min="4" max="4" width="19.5546875" customWidth="1"/>
-    <col min="5" max="5" width="17.33203125" customWidth="1"/>
-    <col min="6" max="6" width="10.33203125" customWidth="1"/>
-    <col min="8" max="8" width="15.44140625" customWidth="1"/>
-    <col min="9" max="9" width="16" customWidth="1"/>
-    <col min="10" max="10" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="24.6640625" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="9.77734375" customWidth="1"/>
+    <col min="7" max="7" width="7.44140625" customWidth="1"/>
+    <col min="8" max="8" width="17.21875" customWidth="1"/>
+    <col min="9" max="9" width="13.21875" customWidth="1"/>
+    <col min="10" max="10" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.88671875" customWidth="1"/>
     <col min="13" max="13" width="15.109375" customWidth="1"/>
     <col min="14" max="14" width="52.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:14" s="30" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="M1" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="N1" s="27" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>27</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>28</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>14</v>
@@ -744,7 +764,7 @@
         <v>0.88</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>17</v>
@@ -759,25 +779,25 @@
       <c r="M2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="N2" s="10" t="s">
+      <c r="N2" s="7" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>30</v>
-      </c>
       <c r="C3" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>15</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>22</v>
@@ -785,163 +805,209 @@
       <c r="G3" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="21" t="s">
-        <v>44</v>
+      <c r="H3" s="23" t="s">
+        <v>43</v>
       </c>
       <c r="I3" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="M3" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="J3" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="M3" s="4" t="s">
+      <c r="N3" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="N3" s="8" t="s">
+    </row>
+    <row r="4" spans="1:14" s="24" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="19" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" s="26" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="D4" s="24"/>
-      <c r="E4" s="25" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="H4" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="I4" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="J4" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="K4" s="23"/>
-      <c r="L4" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="M4" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="N4" s="22" t="s">
-        <v>23</v>
+      <c r="I4" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="J4" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="M4" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="N4" s="18" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="M5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N5" s="10" t="s">
-        <v>25</v>
+      <c r="A5" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="J5" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="K5" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="L5" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="M5" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="N5" s="18" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="C6" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="D6" s="11"/>
+      <c r="E6" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="D6" s="14"/>
-      <c r="E6" s="15" t="s">
+      <c r="J6" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="K6" s="10"/>
+      <c r="L6" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="M6" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="N6" s="13" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="2"/>
+      <c r="E7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="M7" s="25" t="s">
+        <v>22</v>
+      </c>
+      <c r="N7" s="7" t="s">
         <v>24</v>
-      </c>
-      <c r="F6" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="H6" s="13"/>
-      <c r="I6" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="J6" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="K6" s="13"/>
-      <c r="L6" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="M6" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="N6" s="16" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="C9" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="D9" s="20" t="s">
-        <v>41</v>
-      </c>
-      <c r="E9" s="26" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="C10" s="17" t="s">
-        <v>43</v>
-      </c>
-      <c r="D10" s="18" t="s">
+      <c r="C10" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="21" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="C11" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="E10" s="26"/>
+      <c r="D11" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="E11" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updated recall precision and clone types to the excel document
</commit_message>
<xml_diff>
--- a/assignment3/Results.xlsx
+++ b/assignment3/Results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gostg\Documents\vscode\470\CMPT470-Future-Buisness-Majors\assignment3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CBB7755-0FF8-439C-9447-9D650B9B54B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3418C5F4-CBFA-4193-A4C2-DBE9A9C4998D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8670" yWindow="4335" windowWidth="23640" windowHeight="14940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="59">
   <si>
     <t>Tool ID</t>
   </si>
@@ -72,15 +72,9 @@
     <t>default tool settings</t>
   </si>
   <si>
-    <t>Type-1</t>
-  </si>
-  <si>
     <t>Good precision; slight recall drop vs</t>
   </si>
   <si>
-    <t>Cross Language</t>
-  </si>
-  <si>
     <t>N/A</t>
   </si>
   <si>
@@ -193,6 +187,21 @@
   </si>
   <si>
     <t>.88 (varies)</t>
+  </si>
+  <si>
+    <t>0.677 (varies)</t>
+  </si>
+  <si>
+    <t>0.527 (varies)</t>
+  </si>
+  <si>
+    <t>Type 3 (Essence Clones)</t>
+  </si>
+  <si>
+    <t>Type 4 (Semantic Clones)</t>
+  </si>
+  <si>
+    <t>Type 3 &amp; Type 4 Clones</t>
   </si>
 </sst>
 </file>
@@ -252,7 +261,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -277,8 +286,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB4C6E7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -348,6 +363,15 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -361,27 +385,27 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -390,6 +414,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFB4C6E7"/>
       <color rgb="FFFFABAB"/>
       <color rgb="FFFF5B5B"/>
     </mruColors>
@@ -675,7 +700,7 @@
     <col min="2" max="2" width="19.85546875" customWidth="1"/>
     <col min="3" max="3" width="44" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="5" max="5" width="22.7109375" customWidth="1"/>
     <col min="6" max="6" width="9.7109375" customWidth="1"/>
     <col min="7" max="7" width="7.42578125" customWidth="1"/>
     <col min="8" max="8" width="43.42578125" customWidth="1"/>
@@ -688,314 +713,326 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="D1" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="19" t="s">
+      <c r="E1" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="19" t="s">
+      <c r="G1" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="19" t="s">
+      <c r="H1" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="19" t="s">
+      <c r="I1" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="19" t="s">
+      <c r="J1" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="19" t="s">
+      <c r="K1" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="19" t="s">
+      <c r="L1" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="19" t="s">
+      <c r="M1" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="18" t="s">
+      <c r="N1" s="15" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="E2" s="12" t="s">
+      <c r="A2" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="J2" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="K2" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="L2" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="M2" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="N2" s="9" t="s">
         <v>15</v>
-      </c>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="I2" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="M2" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="N2" s="11" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>19</v>
+      <c r="E3" s="26" t="s">
+        <v>57</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="I3" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="J3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="N3" s="5" t="s">
         <v>40</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="N3" s="5" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="G4" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="H4" s="12" t="s">
+      <c r="A4" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="I4" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="I4" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="J4" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="K4" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="L4" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="M4" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="N4" s="11" t="s">
+      <c r="J4" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="K4" s="10" t="s">
         <v>49</v>
+      </c>
+      <c r="L4" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="M4" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="N4" s="9" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="J5" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="K5" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="L5" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="M5" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="N5" s="9" t="s">
         <v>46</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="H5" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="I5" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="J5" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="K5" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="L5" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="M5" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="N5" s="11" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="21" t="s">
-        <v>30</v>
-      </c>
-      <c r="B6" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="25" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" s="24" t="s">
+      <c r="A6" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="F6" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="J6" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="K6" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="L6" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="M6" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="N6" s="18" t="s">
         <v>19</v>
-      </c>
-      <c r="F6" s="23"/>
-      <c r="G6" s="23"/>
-      <c r="H6" s="23" t="s">
-        <v>18</v>
-      </c>
-      <c r="I6" s="23" t="s">
-        <v>45</v>
-      </c>
-      <c r="J6" s="23" t="s">
-        <v>55</v>
-      </c>
-      <c r="K6" s="23" t="s">
-        <v>54</v>
-      </c>
-      <c r="L6" s="23" t="s">
-        <v>18</v>
-      </c>
-      <c r="M6" s="25" t="s">
-        <v>18</v>
-      </c>
-      <c r="N6" s="21" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="K7" s="1"/>
       <c r="L7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="M7" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="N7" s="6" t="s">
         <v>18</v>
-      </c>
-      <c r="M7" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="N7" s="6" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C10" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>44</v>
+      <c r="C10" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="E10" s="24" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C11" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="E11" s="14"/>
+        <v>35</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" s="25"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Actual excel sheet I forgot exists, updated ccdt
</commit_message>
<xml_diff>
--- a/assignment3/Results.xlsx
+++ b/assignment3/Results.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gostg\Documents\vscode\470\CMPT470-Future-Buisness-Majors\assignment3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kylen\gth842\cmpt470-a2\repo\assignment3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{390C7CF0-4D6C-4658-9E87-084D2B5523E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20A8678E-C23E-46B5-80A9-3537DD16144E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="64">
   <si>
     <t>Tool ID</t>
   </si>
@@ -162,12 +162,6 @@
     <t>.891 (varies)</t>
   </si>
   <si>
-    <t>.94 (varies)</t>
-  </si>
-  <si>
-    <t>.88 (varies)</t>
-  </si>
-  <si>
     <t>0.677 (varies)</t>
   </si>
   <si>
@@ -202,12 +196,36 @@
   </si>
   <si>
     <t>Debian 13 /Python 2.7.18 / Java SE 25.0.2</t>
+  </si>
+  <si>
+    <t>Windows 11 / Firefox 148.0.2 / Python 3.14</t>
+  </si>
+  <si>
+    <t>best guess from paper</t>
+  </si>
+  <si>
+    <t>TES E</t>
+  </si>
+  <si>
+    <t>Much worse than expected</t>
+  </si>
+  <si>
+    <t>.880 (varies)</t>
+  </si>
+  <si>
+    <t>.940 (varies)</t>
+  </si>
+  <si>
+    <t>Exact methodology was not stated, had to pre-prompt with educated guess leading to a worse result. Limited to N=50 by hand as OpenAI API is costly.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -373,7 +391,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -394,13 +412,19 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -689,26 +713,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:N10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="46.85546875" customWidth="1"/>
-    <col min="2" max="2" width="19.85546875" customWidth="1"/>
+    <col min="1" max="1" width="46.88671875" customWidth="1"/>
+    <col min="2" max="2" width="27.88671875" customWidth="1"/>
     <col min="3" max="3" width="44" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
-    <col min="5" max="5" width="22.7109375" customWidth="1"/>
-    <col min="6" max="6" width="9.7109375" customWidth="1"/>
-    <col min="7" max="7" width="7.42578125" customWidth="1"/>
-    <col min="8" max="8" width="43.42578125" customWidth="1"/>
-    <col min="9" max="9" width="13.28515625" customWidth="1"/>
-    <col min="10" max="10" width="14.7109375" customWidth="1"/>
-    <col min="11" max="11" width="17.42578125" customWidth="1"/>
-    <col min="12" max="12" width="17.85546875" customWidth="1"/>
-    <col min="13" max="13" width="23.5703125" customWidth="1"/>
-    <col min="14" max="14" width="53" customWidth="1"/>
+    <col min="5" max="5" width="22.6640625" customWidth="1"/>
+    <col min="6" max="6" width="9.6640625" customWidth="1"/>
+    <col min="7" max="7" width="7.44140625" customWidth="1"/>
+    <col min="8" max="8" width="43.44140625" customWidth="1"/>
+    <col min="9" max="9" width="13.33203125" customWidth="1"/>
+    <col min="10" max="10" width="14.6640625" customWidth="1"/>
+    <col min="11" max="11" width="17.44140625" customWidth="1"/>
+    <col min="12" max="12" width="23.77734375" customWidth="1"/>
+    <col min="13" max="13" width="23.5546875" customWidth="1"/>
+    <col min="14" max="14" width="63.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
@@ -752,7 +776,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="13" t="s">
         <v>16</v>
       </c>
@@ -766,7 +790,7 @@
         <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>15</v>
@@ -781,10 +805,10 @@
         <v>36</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="L2" s="6" t="s">
         <v>15</v>
@@ -796,7 +820,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>18</v>
       </c>
@@ -804,13 +828,13 @@
         <v>19</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>14</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>15</v>
@@ -840,7 +864,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>20</v>
       </c>
@@ -854,7 +878,7 @@
         <v>15</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>15</v>
@@ -884,7 +908,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>37</v>
       </c>
@@ -898,7 +922,7 @@
         <v>15</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>15</v>
@@ -928,117 +952,117 @@
         <v>39</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A6" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="F6" s="27">
+        <v>0.182</v>
+      </c>
+      <c r="G6" s="27">
+        <v>0.24299999999999999</v>
+      </c>
+      <c r="H6" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="I6" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="J6" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="K6" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="L6" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="M6" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="N6" s="21" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B7" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="K6" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="L6" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="M6" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="N6" s="5" t="s">
-        <v>39</v>
+      <c r="C7" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" s="26">
+        <v>0.8</v>
+      </c>
+      <c r="G7" s="26">
+        <v>0.6</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="M7" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="N7" s="28" t="s">
+        <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>56</v>
-      </c>
-      <c r="D7" s="21" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="21" t="s">
-        <v>55</v>
-      </c>
-      <c r="F7" s="20">
-        <v>0.182</v>
-      </c>
-      <c r="G7" s="20">
-        <v>0.24299999999999999</v>
-      </c>
-      <c r="H7" s="24" t="s">
-        <v>52</v>
-      </c>
-      <c r="I7" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="J7" s="20" t="s">
-        <v>15</v>
-      </c>
-      <c r="K7" s="20" t="s">
-        <v>15</v>
-      </c>
-      <c r="L7" s="20" t="s">
-        <v>15</v>
-      </c>
-      <c r="M7" s="21" t="s">
-        <v>54</v>
-      </c>
-      <c r="N7" s="22" t="s">
-        <v>57</v>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="C9" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C10" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10" s="15" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C11" s="3" t="s">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="C10" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="D10" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="E11" s="16"/>
+      <c r="E10" s="16"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="H7" r:id="rId1" xr:uid="{E841FCE3-375E-4A6E-9411-5B054FA51EDF}"/>
+    <hyperlink ref="H6" r:id="rId1" xr:uid="{E841FCE3-375E-4A6E-9411-5B054FA51EDF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>